<commit_message>
Planning technicien : colonne Remarque remplacée par Date heure 2nd passage
Format "Lundi 19 octobre 2026 - 08H00 entre 16H00" (le mot "entre"
remplace le tiret entre les deux horaires du 2nd passage, la date
reste séparée par un tiret classique).
</commit_message>
<xml_diff>
--- a/functions/templates/Template-Planning-technicien.xlsx
+++ b/functions/templates/Template-Planning-technicien.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,10 +28,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="12"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -43,10 +46,16 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="9"/>
+      <color rgb="000D1B2A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000D1B2A"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,12 +64,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="000D1B2A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001DA870"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EFEFEF"/>
+        <fgColor rgb="00E8F9F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,33 +88,38 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00D9E2EA"/>
       </left>
       <right style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00D9E2EA"/>
       </right>
       <top style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00D9E2EA"/>
       </top>
       <bottom style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00D9E2EA"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -473,23 +492,24 @@
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>##Nom-fichier</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Belledonne Multiservices</t>
         </is>
       </c>
     </row>
+    <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -497,7 +517,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Adresse</t>
@@ -515,7 +535,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Remarque</t>
+          <t>Date heure 2nd passage</t>
         </is>
       </c>
     </row>
@@ -530,21 +550,22 @@
           <t>##Horaire</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>##NbLogements</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>##Remarque</t>
+          <t>##DateHeure2ndPassage</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Campagnes : colonne Remarque dans les plannings techniciens
Ajoute une colonne "Remarque" (repère ##Remarque) en dernière position du
template Planning technicien, remplie avec la colonne Remarque (G) du
planning source sur la ligne de l'adresse correspondante, vide si absente.
Détection optionnelle : un template sans ##Remarque reste valide.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/functions/templates/Template-Planning-technicien.xlsx
+++ b/functions/templates/Template-Planning-technicien.xlsx
@@ -1,63 +1,105 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25000" windowHeight="10000" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feuille 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet sheetId="1" name="Feuille 1" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+  <si>
+    <t>##Nom-fichier</t>
+  </si>
+  <si>
+    <t>Belledonne Multiservices</t>
+  </si>
+  <si>
+    <t>##Jour-date</t>
+  </si>
+  <si>
+    <t>Adresse</t>
+  </si>
+  <si>
+    <t>Horaire</t>
+  </si>
+  <si>
+    <t>Nb logements</t>
+  </si>
+  <si>
+    <t>Date heure 2nd passage</t>
+  </si>
+  <si>
+    <t>Remarque</t>
+  </si>
+  <si>
+    <t>##Adresse</t>
+  </si>
+  <si>
+    <t>##Horaire</t>
+  </si>
+  <si>
+    <t>##NbLogements</t>
+  </si>
+  <si>
+    <t>##DateHeure2ndPassage</t>
+  </si>
+  <si>
+    <t>##Remarque</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
+      <b/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
+      <name val="Arial"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <i val="1"/>
+      <i/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+      <name val="Arial"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
+      <b/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+      <name val="Arial"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
+      <b/>
       <color rgb="000D1B2A"/>
       <sz val="10"/>
+      <name val="Arial"/>
     </font>
     <font>
-      <name val="Arial"/>
       <color rgb="000D1B2A"/>
       <sz val="10"/>
+      <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -76,6 +118,9 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E8F9F2"/>
       </patternFill>
+    </fill>
+    <fill>
+      <patternFill/>
     </fill>
   </fills>
   <borders count="2">
@@ -99,101 +144,43 @@
       <bottom style="thin">
         <color rgb="00D9E2EA"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -481,91 +468,87 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>##Nom-fichier</t>
-        </is>
-      </c>
+    <row r="1" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
     </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Belledonne Multiservices</t>
-        </is>
-      </c>
+    <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
     </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>##Jour-date</t>
-        </is>
-      </c>
+    <row r="3" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Adresse</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Horaire</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Nb logements</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Date heure 2nd passage</t>
-        </is>
+    <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>##Adresse</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>##Horaire</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>##NbLogements</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>##DateHeure2ndPassage</t>
-        </is>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A4:E4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>